<commit_message>
format and second round
</commit_message>
<xml_diff>
--- a/march-madness-tracker/public/march.xlsx
+++ b/march-madness-tracker/public/march.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="115">
   <si>
     <t>3/19/2026 - First Round</t>
   </si>
@@ -280,19 +280,43 @@
     <t>Missouri</t>
   </si>
   <si>
-    <t>Miami</t>
+    <t>Miami (Fla.)</t>
   </si>
   <si>
     <t>3/21/2026 - Second Round</t>
+  </si>
+  <si>
+    <t>(1) Duke vs. (9) TCU | 5:15 p.m. | CBS</t>
+  </si>
+  <si>
+    <t>(3) Michigan State vs. (6) Louisville | 2:45 p.m. | CBS</t>
+  </si>
+  <si>
+    <t>(4) Arkansas vs. (12) High Point | 9:45 p.m. | TBS</t>
+  </si>
+  <si>
+    <t>(3) Gonzaga (11) Texas | 7:10 p.m. | TBS</t>
+  </si>
+  <si>
+    <t>(4) Nebraska vs. (5) Vanderbilt | 8:45 p.m. | TNT</t>
+  </si>
+  <si>
+    <t>(3) Illinois vs. (11) VCU | 7:50 p.m. | CBS</t>
+  </si>
+  <si>
+    <t>(2) Houston vs. (10) Texas A&amp;M | 6:10 p.m. | TNT</t>
+  </si>
+  <si>
+    <t>(1) Michigan vs. (9) Saint Louis | 12:10 p.m. | CBS</t>
+  </si>
+  <si>
+    <t>3/22/2026 - Second Round</t>
   </si>
   <si>
     <t>Game 1</t>
   </si>
   <si>
     <t xml:space="preserve">Game 2 </t>
-  </si>
-  <si>
-    <t>KU</t>
   </si>
   <si>
     <t>Game 3</t>
@@ -304,6 +328,9 @@
     <t>Game 5</t>
   </si>
   <si>
+    <t>KU</t>
+  </si>
+  <si>
     <t>Game 6</t>
   </si>
   <si>
@@ -311,9 +338,6 @@
   </si>
   <si>
     <t>Game 8</t>
-  </si>
-  <si>
-    <t>3/22/2026 - Second Round</t>
   </si>
   <si>
     <t>3/26/2026 - Sweet 16</t>
@@ -338,7 +362,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -348,6 +372,11 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Open Sans&quot;"/>
     </font>
   </fonts>
   <fills count="2">
@@ -364,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -376,6 +405,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2329,16 +2361,6 @@
       <c r="I40" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2"/>
-      <c r="P40" s="2"/>
-      <c r="Q40" s="2"/>
-      <c r="R40" s="2"/>
-      <c r="S40" s="2"/>
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
@@ -2348,7 +2370,7 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B41" s="3" t="s">
@@ -2375,16 +2397,6 @@
       <c r="I41" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" s="2"/>
-      <c r="Q41" s="2"/>
-      <c r="R41" s="2"/>
-      <c r="S41" s="2"/>
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
@@ -2394,43 +2406,33 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="4" t="s">
         <v>92</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-      <c r="R42" s="2"/>
-      <c r="S42" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="T42" s="2"/>
       <c r="U42" s="2"/>
       <c r="V42" s="2"/>
@@ -2440,43 +2442,33 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="s">
-        <v>94</v>
+      <c r="A43" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
-      <c r="P43" s="2"/>
-      <c r="Q43" s="2"/>
-      <c r="R43" s="2"/>
-      <c r="S43" s="2"/>
+        <v>28</v>
+      </c>
       <c r="T43" s="2"/>
       <c r="U43" s="2"/>
       <c r="V43" s="2"/>
@@ -2486,34 +2478,33 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="s">
-        <v>95</v>
+      <c r="A44" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>86</v>
+        <v>35</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="J44" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
@@ -2532,34 +2523,33 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>57</v>
+      <c r="A45" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J45" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
@@ -2578,34 +2568,33 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>28</v>
+      <c r="A46" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J46" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>41</v>
+      </c>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -2624,34 +2613,33 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>35</v>
+      <c r="A47" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>35</v>
+        <v>48</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="J47" s="2"/>
+        <v>48</v>
+      </c>
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
@@ -2670,32 +2658,32 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>79</v>
+      <c r="A48" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>79</v>
+        <v>33</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -2773,7 +2761,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>1</v>
@@ -2819,7 +2807,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>81</v>
@@ -2865,31 +2853,31 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>13</v>
+        <v>79</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -2911,31 +2899,31 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -2957,31 +2945,31 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>48</v>
+        <v>103</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>48</v>
+        <v>86</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>48</v>
+        <v>77</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I55" s="3" t="s">
-        <v>48</v>
+        <v>77</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
@@ -3003,31 +2991,31 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>33</v>
+        <v>104</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -3049,7 +3037,7 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>54</v>
@@ -3095,7 +3083,7 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>59</v>
@@ -3141,7 +3129,7 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>61</v>
@@ -3215,7 +3203,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>1</v>
@@ -3261,7 +3249,7 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>22</v>
@@ -3307,7 +3295,7 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>86</v>
@@ -3353,7 +3341,7 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>57</v>
@@ -3399,7 +3387,7 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>79</v>
@@ -3473,7 +3461,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>1</v>
@@ -3519,7 +3507,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>24</v>
@@ -3565,7 +3553,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>48</v>
@@ -3611,7 +3599,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>33</v>
@@ -3657,7 +3645,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>61</v>
@@ -3722,7 +3710,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>1</v>
@@ -3768,7 +3756,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>48</v>
@@ -3814,7 +3802,7 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>33</v>
@@ -3916,7 +3904,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>1</v>
@@ -3962,7 +3950,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>86</v>
@@ -4008,7 +3996,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>57</v>
@@ -4082,7 +4070,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>1</v>
@@ -4128,7 +4116,7 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>48</v>
@@ -4174,7 +4162,7 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>57</v>
@@ -4248,7 +4236,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>1</v>
@@ -4294,7 +4282,7 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>48</v>

</xml_diff>